<commit_message>
Rename electricity timeslices in EPS subscript, variable names, and input data files (issue #413)
</commit_message>
<xml_diff>
--- a/InputData/elec/ELCCAfR/ELCCAfR Effective Load Carrying Capability Adjustment for Reliability.xlsx
+++ b/InputData/elec/ELCCAfR/ELCCAfR Effective Load Carrying Capability Adjustment for Reliability.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\ELCCAfR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6617014E-0B48-458E-B9D8-C8AD3BBCCFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2339A624-4442-4DFE-AC1E-EED06727FEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -308,24 +308,6 @@
     <t>Hour23</t>
   </si>
   <si>
-    <t>Winter</t>
-  </si>
-  <si>
-    <t>Spring</t>
-  </si>
-  <si>
-    <t>Summer</t>
-  </si>
-  <si>
-    <t>Fall</t>
-  </si>
-  <si>
-    <t>Summer Peak</t>
-  </si>
-  <si>
-    <t>Winter Peak</t>
-  </si>
-  <si>
     <t>solar thermal</t>
   </si>
   <si>
@@ -510,6 +492,24 @@
   </si>
   <si>
     <t>DRAFT for review. 0.98 for every firm/dispatchable source except hydro (fossil, nuclear, SMR, biomass, MSW, geothermal, CCS and hydrogen types); hydro stays at 0.90 because its derate reflects water limits, not forced outages. For MCF-path plants the reliability credit is MCF x RAF x ELCCAfR, so forced outages and regional availability are already derated by MCF (0.85-0.95) and RAF before this factor applies. At the previous 0.90, the combined credit for gas combined cycle and steam turbines was 0.77, below the NERC GADS 1-EFORd class averages of 0.89-0.95 (2020-2024), which counted outage risk twice. At 0.98 it is 0.84, still at or below those benchmarks, so ELCCAfR now covers only residual risks not captured in MCF or RAF, such as ambient-temperature derates at the summer peak and common-mode fuel-supply risk. Nuclear, SMR, biomass, MSW and geothermal are on the SYSHECF path, so their combined credit is SYSHECF-based; nuclear remains below its 0.975-0.984 benchmark. Arithmetic on the Thermal-derivation tab. Value from Robbie's sandbox setting (2026-09-30); rationale drafted from the NERC GADS benchmarks and pending Robbie's review.</t>
+  </si>
+  <si>
+    <t>Representative Day 1</t>
+  </si>
+  <si>
+    <t>Representative Day 2</t>
+  </si>
+  <si>
+    <t>Representative Day 3</t>
+  </si>
+  <si>
+    <t>Representative Day 4</t>
+  </si>
+  <si>
+    <t>Net Peak Summer Day</t>
+  </si>
+  <si>
+    <t>Net Peak Winter Day</t>
   </si>
 </sst>
 </file>
@@ -1189,7 +1189,7 @@
     <row r="27" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="12" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -1250,7 +1250,7 @@
     <row r="34" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="12" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
@@ -1390,7 +1390,7 @@
     </row>
     <row r="49" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>40</v>
@@ -1419,10 +1419,10 @@
     </row>
     <row r="52" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C52" s="10"/>
       <c r="D52" s="10"/>
@@ -1430,10 +1430,10 @@
     </row>
     <row r="53" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="10"/>
@@ -1604,7 +1604,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -1681,7 +1681,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -1782,7 +1782,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -1984,7 +1984,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2085,7 +2085,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2186,7 +2186,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2303,7 +2303,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -2380,7 +2380,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2481,7 +2481,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2582,7 +2582,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2683,7 +2683,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2784,7 +2784,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -2885,7 +2885,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3002,7 +3002,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -3079,7 +3079,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3180,7 +3180,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3281,7 +3281,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3382,7 +3382,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3483,7 +3483,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3584,7 +3584,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3701,7 +3701,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -3778,7 +3778,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3879,7 +3879,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -3980,7 +3980,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4081,7 +4081,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4182,7 +4182,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4283,7 +4283,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4400,7 +4400,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -4477,7 +4477,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4578,7 +4578,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4679,7 +4679,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4780,7 +4780,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4881,7 +4881,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -4982,7 +4982,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -5099,7 +5099,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -5176,7 +5176,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'DAT-derivation'!$B$24</f>
@@ -5277,7 +5277,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'DAT-derivation'!$B$24</f>
@@ -5378,7 +5378,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'DAT-derivation'!$B$24</f>
@@ -5479,7 +5479,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'DAT-derivation'!$B$24</f>
@@ -5580,7 +5580,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'DAT-derivation'!$B$24</f>
@@ -5681,7 +5681,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'DAT-derivation'!$B$24</f>
@@ -5798,7 +5798,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -5875,7 +5875,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -5976,7 +5976,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6077,7 +6077,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6178,7 +6178,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6279,7 +6279,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6380,7 +6380,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6497,7 +6497,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -6574,7 +6574,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6675,7 +6675,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6776,7 +6776,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6877,7 +6877,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -6978,7 +6978,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7079,7 +7079,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7196,7 +7196,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -7273,7 +7273,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7374,7 +7374,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7475,7 +7475,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7576,7 +7576,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7677,7 +7677,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7778,7 +7778,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -7895,7 +7895,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -7972,7 +7972,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -8073,7 +8073,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -8174,7 +8174,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -8275,7 +8275,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -8376,7 +8376,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -8477,7 +8477,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -8594,7 +8594,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -8698,7 +8698,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B13">
         <f>ROUND(B12,2)</f>
@@ -8717,12 +8717,12 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B20">
         <v>0.45</v>
@@ -8730,7 +8730,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B21">
         <v>0.55000000000000004</v>
@@ -8738,7 +8738,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B22">
         <v>0.8</v>
@@ -8746,7 +8746,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B23">
         <v>0.95</v>
@@ -8754,7 +8754,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B24">
         <v>0.82</v>
@@ -8762,7 +8762,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B25">
         <f>B20*B24</f>
@@ -8771,7 +8771,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B26">
         <f>B21*B24</f>
@@ -8780,12 +8780,12 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -8806,7 +8806,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -8883,7 +8883,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <v>0.9</v>
@@ -8960,7 +8960,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <v>0.9</v>
@@ -9037,7 +9037,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <v>0.9</v>
@@ -9114,7 +9114,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <v>0.9</v>
@@ -9191,7 +9191,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <v>0.9</v>
@@ -9268,7 +9268,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <v>0.9</v>
@@ -9361,7 +9361,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -9438,7 +9438,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -9539,7 +9539,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -9640,7 +9640,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -9741,7 +9741,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -9842,7 +9842,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -9943,7 +9943,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10060,7 +10060,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -10137,7 +10137,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10238,7 +10238,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10339,7 +10339,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10440,7 +10440,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10541,7 +10541,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10642,7 +10642,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10759,7 +10759,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -10836,7 +10836,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -10937,7 +10937,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11038,7 +11038,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11139,7 +11139,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11240,7 +11240,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11341,7 +11341,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11458,7 +11458,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -11535,7 +11535,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11636,7 +11636,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11737,7 +11737,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11838,7 +11838,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -11939,7 +11939,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12040,7 +12040,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12157,7 +12157,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -12234,7 +12234,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12335,7 +12335,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12436,7 +12436,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12537,7 +12537,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12638,7 +12638,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12739,7 +12739,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -12856,7 +12856,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -12933,7 +12933,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13034,7 +13034,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13135,7 +13135,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13236,7 +13236,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13337,7 +13337,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13438,7 +13438,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13555,7 +13555,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -13632,7 +13632,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13733,7 +13733,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13834,7 +13834,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -13935,7 +13935,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14036,7 +14036,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14137,7 +14137,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14254,7 +14254,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -14331,7 +14331,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14432,7 +14432,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14533,7 +14533,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14634,7 +14634,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14735,7 +14735,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14836,7 +14836,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -14951,12 +14951,12 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B3">
         <v>0.98</v>
@@ -14964,7 +14964,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B4">
         <v>0.9</v>
@@ -14972,32 +14972,32 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B8" s="15">
         <v>0.95</v>
@@ -15019,7 +15019,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B9" s="15">
         <v>0.95</v>
@@ -15036,12 +15036,12 @@
         <v>0.83789999999999998</v>
       </c>
       <c r="F9" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B10" s="15">
         <v>0.95</v>
@@ -15058,12 +15058,12 @@
         <v>0.83789999999999998</v>
       </c>
       <c r="F10" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B11" s="15">
         <v>0.85</v>
@@ -15080,12 +15080,12 @@
         <v>0.52478999999999998</v>
       </c>
       <c r="F11" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B12" s="15">
         <v>0.95</v>
@@ -15102,32 +15102,32 @@
         <v>0.74480000000000002</v>
       </c>
       <c r="F12" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -15226,7 +15226,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2" s="5">
         <v>1</v>
@@ -15303,7 +15303,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
@@ -15380,7 +15380,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
@@ -15457,7 +15457,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5" s="5">
         <v>1</v>
@@ -15534,7 +15534,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6" s="5">
         <v>1</v>
@@ -15611,7 +15611,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7" s="5">
         <v>1</v>
@@ -15705,7 +15705,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>58</v>
@@ -15782,7 +15782,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2" s="5">
         <v>1</v>
@@ -15859,7 +15859,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
@@ -15936,7 +15936,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
@@ -16013,7 +16013,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5" s="5">
         <v>1</v>
@@ -16090,7 +16090,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6" s="5">
         <v>1</v>
@@ -16167,7 +16167,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7" s="5">
         <v>1</v>
@@ -16261,7 +16261,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>58</v>
@@ -16338,7 +16338,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2" s="5">
         <v>1</v>
@@ -16415,7 +16415,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
@@ -16492,7 +16492,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
@@ -16569,7 +16569,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5" s="5">
         <v>1</v>
@@ -16646,7 +16646,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6" s="7">
         <v>0.80869999999999997</v>
@@ -16723,7 +16723,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7" s="7">
         <v>0.69359999999999999</v>
@@ -16817,7 +16817,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>58</v>
@@ -16894,7 +16894,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2" s="5">
         <v>1</v>
@@ -16971,7 +16971,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
@@ -17048,7 +17048,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
@@ -17125,7 +17125,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5" s="5">
         <v>1</v>
@@ -17202,7 +17202,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6" s="7">
         <v>0.3342</v>
@@ -17279,7 +17279,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7" s="7">
         <v>0.85509999999999997</v>
@@ -17372,7 +17372,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -17449,7 +17449,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -17550,7 +17550,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -17651,7 +17651,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -17752,7 +17752,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -17853,7 +17853,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -17954,7 +17954,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>
@@ -18071,7 +18071,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>58</v>
@@ -18148,7 +18148,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <f>'Thermal-derivation'!$B$3</f>
@@ -18249,7 +18249,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="B3">
         <f>'Thermal-derivation'!$B$3</f>
@@ -18350,7 +18350,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <f>'Thermal-derivation'!$B$3</f>
@@ -18451,7 +18451,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <f>'Thermal-derivation'!$B$3</f>
@@ -18552,7 +18552,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <f>'Thermal-derivation'!$B$3</f>
@@ -18653,7 +18653,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <f>'Thermal-derivation'!$B$3</f>

</xml_diff>